<commit_message>
Update badges and use the permanent Zenodo DOI
DOI badge points to concept DOI 10.5281/zenodo.3976631, Tests badge
added, lifecycle moves from maturing (retired stage) to stable. DOI
added to CITATION.cff, the metadata sheet and the CFF helper.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LpE9sX4VLC7ZBF4MdDbNUP
</commit_message>
<xml_diff>
--- a/metadata/project-metadata.xlsx
+++ b/metadata/project-metadata.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -635,6 +635,18 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>agriculture; digital innovation; FAIR data; partnerships for the goals; tricot approach</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>doi</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.3976631</t>
         </is>
       </c>
     </row>

</xml_diff>